<commit_message>
Add uploaded OCHA figures (Excel) for Haiti___HTI
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Haiti___HTI/ocha_figures_Haiti___HTI_1021_04PM.xlsx
+++ b/platform_PiN_output/Haiti___HTI/ocha_figures_Haiti___HTI_1021_04PM.xlsx
@@ -5397,7 +5397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HT0121</t>
+          <t>HT0115</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HT0122</t>
+          <t>HT0116</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HT0123</t>
+          <t>HT0121</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HT0132</t>
+          <t>HT0122</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HT0134</t>
+          <t>HT0123</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HT0135</t>
+          <t>HT0132</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HT0141</t>
+          <t>HT0133</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5540,7 +5540,7 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HT0142</t>
+          <t>HT0134</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5553,7 +5553,7 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HT0151</t>
+          <t>HT0135</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5566,7 +5566,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HT0152</t>
+          <t>HT0141</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5579,7 +5579,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HT0211</t>
+          <t>HT0142</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -5588,7 +5588,7 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HT0212</t>
+          <t>HT0151</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -5597,7 +5597,7 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HT0214</t>
+          <t>HT0152</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -5606,7 +5606,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HT0221</t>
+          <t>HT0211</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -5615,7 +5615,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HT0222</t>
+          <t>HT0212</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -5624,7 +5624,7 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HT0231</t>
+          <t>HT0213</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -5633,7 +5633,7 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HT0232</t>
+          <t>HT0214</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -5642,7 +5642,7 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HT0233</t>
+          <t>HT0221</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -5651,7 +5651,7 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HT0234</t>
+          <t>HT0222</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -5660,7 +5660,7 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HT0311</t>
+          <t>HT0231</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -5669,7 +5669,7 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HT0313</t>
+          <t>HT0232</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -5678,7 +5678,7 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HT0321</t>
+          <t>HT0233</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -5687,7 +5687,7 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HT0322</t>
+          <t>HT0234</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -5696,7 +5696,7 @@
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HT0323</t>
+          <t>HT0311</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -5705,7 +5705,7 @@
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HT0331</t>
+          <t>HT0312</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -5714,7 +5714,7 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HT0332</t>
+          <t>HT0313</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -5723,7 +5723,7 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HT0341</t>
+          <t>HT0321</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -5732,7 +5732,7 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>HT0342</t>
+          <t>HT0322</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -5741,7 +5741,7 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HT0343</t>
+          <t>HT0323</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -5750,7 +5750,7 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>HT0344</t>
+          <t>HT0331</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -5759,7 +5759,7 @@
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HT0351</t>
+          <t>HT0332</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -5768,7 +5768,7 @@
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HT0352</t>
+          <t>HT0341</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -5777,7 +5777,7 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HT0361</t>
+          <t>HT0342</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -5786,7 +5786,7 @@
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HT0371</t>
+          <t>HT0343</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -5795,7 +5795,7 @@
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HT0372</t>
+          <t>HT0344</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -5804,7 +5804,7 @@
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HT0411</t>
+          <t>HT0345</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -5813,7 +5813,7 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>HT0412</t>
+          <t>HT0351</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -5822,7 +5822,7 @@
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HT0413</t>
+          <t>HT0352</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -5831,7 +5831,7 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HT0421</t>
+          <t>HT0361</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -5840,7 +5840,7 @@
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
-          <t>HT0422</t>
+          <t>HT0362</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -5849,7 +5849,7 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
-          <t>HT0423</t>
+          <t>HT0371</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -5858,7 +5858,7 @@
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>HT0431</t>
+          <t>HT0372</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -5867,7 +5867,7 @@
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
-          <t>HT0432</t>
+          <t>HT0411</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -5876,7 +5876,7 @@
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
-          <t>HT0433</t>
+          <t>HT0412</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -5885,7 +5885,7 @@
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
-          <t>HT0441</t>
+          <t>HT0413</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -5894,7 +5894,7 @@
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
-          <t>HT0442</t>
+          <t>HT0421</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -5903,7 +5903,7 @@
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
-          <t>HT0443</t>
+          <t>HT0422</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -5912,7 +5912,7 @@
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
-          <t>HT0511</t>
+          <t>HT0423</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -5921,7 +5921,7 @@
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HT0512</t>
+          <t>HT0431</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -5930,7 +5930,7 @@
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HT0521</t>
+          <t>HT0432</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -5939,7 +5939,7 @@
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HT0522</t>
+          <t>HT0433</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -5948,7 +5948,7 @@
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
-          <t>HT0523</t>
+          <t>HT0434</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -5957,7 +5957,7 @@
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
-          <t>HT0531</t>
+          <t>HT0441</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -5966,7 +5966,7 @@
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
-          <t>HT0532</t>
+          <t>HT0442</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -5975,7 +5975,7 @@
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
-          <t>HT0541</t>
+          <t>HT0443</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -5984,7 +5984,7 @@
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
-          <t>HT0551</t>
+          <t>HT0511</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -5993,7 +5993,7 @@
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
-          <t>HT0552</t>
+          <t>HT0512</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -6002,7 +6002,7 @@
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
-          <t>HT0611</t>
+          <t>HT0513</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -6011,7 +6011,7 @@
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
-          <t>HT0612</t>
+          <t>HT0521</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -6020,7 +6020,7 @@
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
-          <t>HT0613</t>
+          <t>HT0522</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -6029,7 +6029,7 @@
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
-          <t>HT0614</t>
+          <t>HT0523</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -6038,7 +6038,7 @@
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
-          <t>HT0621</t>
+          <t>HT0531</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -6047,7 +6047,7 @@
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
-          <t>HT0623</t>
+          <t>HT0532</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -6056,7 +6056,7 @@
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
-          <t>HT0631</t>
+          <t>HT0533</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -6065,7 +6065,7 @@
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
-          <t>HT0632</t>
+          <t>HT0541</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -6074,7 +6074,7 @@
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
-          <t>HT0633</t>
+          <t>HT0542</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -6083,7 +6083,7 @@
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
-          <t>HT0641</t>
+          <t>HT0543</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -6092,7 +6092,7 @@
       <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
-          <t>HT0642</t>
+          <t>HT0544</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -6101,7 +6101,7 @@
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
-          <t>HT0711</t>
+          <t>HT0551</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -6110,7 +6110,7 @@
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
-          <t>HT0712</t>
+          <t>HT0552</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -6119,7 +6119,7 @@
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
-          <t>HT0713</t>
+          <t>HT0611</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -6128,7 +6128,7 @@
       <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
-          <t>HT0714</t>
+          <t>HT0612</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -6137,7 +6137,7 @@
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
-          <t>HT0715</t>
+          <t>HT0613</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -6146,7 +6146,7 @@
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
-          <t>HT0721</t>
+          <t>HT0614</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -6155,7 +6155,7 @@
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
-          <t>HT0722</t>
+          <t>HT0621</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -6164,7 +6164,7 @@
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
-          <t>HT0731</t>
+          <t>HT0622</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -6173,7 +6173,7 @@
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
-          <t>HT0732</t>
+          <t>HT0623</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -6182,7 +6182,7 @@
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
-          <t>HT0733</t>
+          <t>HT0631</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -6191,7 +6191,7 @@
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
-          <t>HT0741</t>
+          <t>HT0632</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -6200,7 +6200,7 @@
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
-          <t>HT0742</t>
+          <t>HT0633</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -6209,7 +6209,7 @@
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
-          <t>HT0743</t>
+          <t>HT0641</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -6218,7 +6218,7 @@
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
-          <t>HT0751</t>
+          <t>HT0642</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
@@ -6227,7 +6227,7 @@
       <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
-          <t>HT0753</t>
+          <t>HT0711</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -6236,7 +6236,7 @@
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
-          <t>HT0811</t>
+          <t>HT0712</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -6245,7 +6245,7 @@
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
-          <t>HT0812</t>
+          <t>HT0713</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -6254,7 +6254,7 @@
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
-          <t>HT0814</t>
+          <t>HT0714</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -6263,7 +6263,7 @@
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
-          <t>HT0821</t>
+          <t>HT0715</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
@@ -6272,7 +6272,7 @@
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
-          <t>HT0822</t>
+          <t>HT0716</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
@@ -6281,7 +6281,7 @@
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
-          <t>HT0823</t>
+          <t>HT0721</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -6290,7 +6290,7 @@
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
-          <t>HT0831</t>
+          <t>HT0722</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6299,7 +6299,7 @@
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
-          <t>HT0832</t>
+          <t>HT0723</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
@@ -6308,7 +6308,7 @@
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
-          <t>HT0833</t>
+          <t>HT0731</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6317,7 +6317,7 @@
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
-          <t>HT0834</t>
+          <t>HT0732</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6326,7 +6326,7 @@
       <c r="A95" t="inlineStr"/>
       <c r="B95" t="inlineStr">
         <is>
-          <t>HT0911</t>
+          <t>HT0733</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -6335,7 +6335,7 @@
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr">
         <is>
-          <t>HT0912</t>
+          <t>HT0741</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -6344,7 +6344,7 @@
       <c r="A97" t="inlineStr"/>
       <c r="B97" t="inlineStr">
         <is>
-          <t>HT0913</t>
+          <t>HT0742</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -6353,7 +6353,7 @@
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="inlineStr">
         <is>
-          <t>HT0914</t>
+          <t>HT0743</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -6362,7 +6362,7 @@
       <c r="A99" t="inlineStr"/>
       <c r="B99" t="inlineStr">
         <is>
-          <t>HT0921</t>
+          <t>HT0751</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -6371,7 +6371,7 @@
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="inlineStr">
         <is>
-          <t>HT0922</t>
+          <t>HT0752</t>
         </is>
       </c>
       <c r="C100" t="inlineStr"/>
@@ -6380,7 +6380,7 @@
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="inlineStr">
         <is>
-          <t>HT0931</t>
+          <t>HT0753</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -6389,7 +6389,7 @@
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="inlineStr">
         <is>
-          <t>HT0932</t>
+          <t>HT0811</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
@@ -6398,7 +6398,7 @@
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="inlineStr">
         <is>
-          <t>HT0934</t>
+          <t>HT0812</t>
         </is>
       </c>
       <c r="C103" t="inlineStr"/>
@@ -6407,7 +6407,7 @@
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="inlineStr">
         <is>
-          <t>HT1011</t>
+          <t>HT0813</t>
         </is>
       </c>
       <c r="C104" t="inlineStr"/>
@@ -6416,7 +6416,7 @@
       <c r="A105" t="inlineStr"/>
       <c r="B105" t="inlineStr">
         <is>
-          <t>HT1012</t>
+          <t>HT0814</t>
         </is>
       </c>
       <c r="C105" t="inlineStr"/>
@@ -6425,7 +6425,7 @@
       <c r="A106" t="inlineStr"/>
       <c r="B106" t="inlineStr">
         <is>
-          <t>HT1013</t>
+          <t>HT0815</t>
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
@@ -6434,7 +6434,7 @@
       <c r="A107" t="inlineStr"/>
       <c r="B107" t="inlineStr">
         <is>
-          <t>HT1014</t>
+          <t>HT0821</t>
         </is>
       </c>
       <c r="C107" t="inlineStr"/>
@@ -6443,7 +6443,7 @@
       <c r="A108" t="inlineStr"/>
       <c r="B108" t="inlineStr">
         <is>
-          <t>HT1021</t>
+          <t>HT0822</t>
         </is>
       </c>
       <c r="C108" t="inlineStr"/>
@@ -6452,7 +6452,7 @@
       <c r="A109" t="inlineStr"/>
       <c r="B109" t="inlineStr">
         <is>
-          <t>HT1022</t>
+          <t>HT0823</t>
         </is>
       </c>
       <c r="C109" t="inlineStr"/>
@@ -6461,7 +6461,7 @@
       <c r="A110" t="inlineStr"/>
       <c r="B110" t="inlineStr">
         <is>
-          <t>HT1023</t>
+          <t>HT0831</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -6470,7 +6470,7 @@
       <c r="A111" t="inlineStr"/>
       <c r="B111" t="inlineStr">
         <is>
-          <t>HT1024</t>
+          <t>HT0832</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
@@ -6479,7 +6479,7 @@
       <c r="A112" t="inlineStr"/>
       <c r="B112" t="inlineStr">
         <is>
-          <t>HT1025</t>
+          <t>HT0833</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -6488,7 +6488,7 @@
       <c r="A113" t="inlineStr"/>
       <c r="B113" t="inlineStr">
         <is>
-          <t>HT1031</t>
+          <t>HT0834</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
@@ -6497,10 +6497,190 @@
       <c r="A114" t="inlineStr"/>
       <c r="B114" t="inlineStr">
         <is>
+          <t>HT0911</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr"/>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>HT0912</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr"/>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>HT0913</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr"/>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>HT0914</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr"/>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HT0921</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>HT0922</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr"/>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>HT0931</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr"/>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>HT0932</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr"/>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>HT0933</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr"/>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>HT0934</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr"/>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>HT1011</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr"/>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>HT1012</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr"/>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>HT1013</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr"/>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>HT1014</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr"/>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>HT1021</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr"/>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>HT1022</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr"/>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>HT1023</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr"/>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>HT1024</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr"/>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>HT1025</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr"/>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>HT1031</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr"/>
+      <c r="B134" t="inlineStr">
+        <is>
           <t>HT1032</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
+      <c r="C134" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>